<commit_message>
feat: add client-scoped order workflows and tracking operations
Add Client/Sales access controls, service settings, purchase queue, shipment status, bulk tracking replacements and order audit history. Preserve legacy accounts and migrate tracking charge references without duplicate debits.

Include regression checks for access control, order calculations, API workflows, imports and legacy migration. Local verification: 147 assertions passed and production webpack build succeeded. Browser UI and live Jenkins deployment remain unverified; cancellation and Client-specific Balance imports remain pending.
</commit_message>
<xml_diff>
--- a/public/templates/dmd-admin-orders.xlsx
+++ b/public/templates/dmd-admin-orders.xlsx
@@ -16,9 +16,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
-    <t>Ngày tạo</t>
-  </si>
-  <si>
     <t>Sales</t>
   </si>
   <si>
@@ -40,7 +37,7 @@
     <t>Tracking</t>
   </si>
   <si>
-    <t>Order ID</t>
+    <t>Client Order ID</t>
   </si>
   <si>
     <t>Net Cost</t>
@@ -55,6 +52,9 @@
     <t>Discount</t>
   </si>
   <si>
+    <t>Lý do Discount</t>
+  </si>
+  <si>
     <t>Sales Price</t>
   </si>
   <si>
@@ -124,7 +124,7 @@
     <t>Điện thoại</t>
   </si>
   <si>
-    <t>RULE: Không đổi tên cột. Sales nên khớp Display Name hoặc Username của account đang Active.</t>
+    <t>RULE: Không đổi tên cột. Client Order ID là mã do khách cung cấp; DMD ID do hệ thống tự sinh. Ngày tạo do hệ thống tự lưu. Sales nên khớp Display Name hoặc Username đang Active.</t>
   </si>
 </sst>
 </file>

</xml_diff>